<commit_message>
new run (091024), implemented plot_mean in plot_drc
</commit_message>
<xml_diff>
--- a/plate_layout_gi50.xlsx
+++ b/plate_layout_gi50.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s1754085\Documents\GitProjects\drc_analyser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FA838EE-14AB-481D-B741-1EBA2456A62D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196AACC8-CA29-45B6-B791-F3B817C0954D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="3" xr2:uid="{8FCF5819-8A68-4587-A348-706285528510}"/>
+    <workbookView xWindow="38280" yWindow="1260" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{8FCF5819-8A68-4587-A348-706285528510}"/>
   </bookViews>
   <sheets>
     <sheet name="help" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="17">
   <si>
     <t>A</t>
   </si>
@@ -1518,6 +1518,30 @@
       <c r="B5" t="s">
         <v>9</v>
       </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" t="s">
+        <v>16</v>
+      </c>
       <c r="M5" t="s">
         <v>9</v>
       </c>

</xml_diff>